<commit_message>
Update Pemetaan Posisi / Role
BCP, TODJO, dan DJK Service
</commit_message>
<xml_diff>
--- a/Daily mp-v10/skills/daily-mp/references/Detail_SCs.xlsx
+++ b/Daily mp-v10/skills/daily-mp/references/Detail_SCs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MDhaniWidoyoko\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2. Download\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{150BBAFD-564C-4618-818C-45554FC9AAD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31AC3A8E-DA63-4240-87FF-072B01C5F7D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14505" yWindow="-4635" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pemetaan Posisi" sheetId="1" r:id="rId1"/>
@@ -29,8 +29,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -38,7 +36,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -60,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="196">
   <si>
     <t>DHJ</t>
   </si>
@@ -284,9 +282,6 @@
     <t>Land 1</t>
   </si>
   <si>
-    <t>Team Electrical, Team 5R HSE, Night Shift</t>
-  </si>
-  <si>
     <t>Engineering Department</t>
   </si>
   <si>
@@ -299,9 +294,6 @@
     <t>eng</t>
   </si>
   <si>
-    <t>Land 2 (Warehouse)</t>
-  </si>
-  <si>
     <t>SPV Matecon</t>
   </si>
   <si>
@@ -621,6 +613,39 @@
   </si>
   <si>
     <t>Fitter, Skill, Welder</t>
+  </si>
+  <si>
+    <t>Team Electrical M&amp;E, Team 5R HSE, Team 5R GA, Night Shift.</t>
+  </si>
+  <si>
+    <t>Day Shift Land 2 (Warehouse)</t>
+  </si>
+  <si>
+    <t>SE</t>
+  </si>
+  <si>
+    <t>HSE Koord, HSE Coordinator, HSE Officer, HSE</t>
+  </si>
+  <si>
+    <t>Surveyor, Ass Surveyor, Survey</t>
+  </si>
+  <si>
+    <t>QC, QC Checker</t>
+  </si>
+  <si>
+    <t>Insp Scaff, Inspector Scaffolder, Scaffolder</t>
+  </si>
+  <si>
+    <t>Rigger, Fitter</t>
+  </si>
+  <si>
+    <t>Admin, Matkon, Material Control</t>
+  </si>
+  <si>
+    <t>PM, SM</t>
+  </si>
+  <si>
+    <t>Busbar, Teknisi, Wiring</t>
   </si>
 </sst>
 </file>
@@ -641,6 +666,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1110,26 +1136,26 @@
     </row>
     <row r="9" spans="1:9" ht="12.75">
       <c r="A9" s="26" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C9" s="25"/>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" ht="12.75">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
     </row>
     <row r="11" spans="1:9" ht="12.75">
       <c r="A11" s="28" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B11" s="5"/>
     </row>
     <row r="12" spans="1:9" ht="12.75">
       <c r="A12" s="18" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B12" s="18" t="str" cm="1">
         <f t="array" ref="B12:H12">TRANSPOSE(A2:A8)</f>
@@ -1154,7 +1180,7 @@
         <v>TODJO</v>
       </c>
       <c r="I12" s="20" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="12.75">
@@ -1214,10 +1240,14 @@
         <v>22</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>153</v>
-      </c>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
+        <v>151</v>
+      </c>
+      <c r="G15" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="H15" s="16" t="s">
+        <v>151</v>
+      </c>
       <c r="I15" s="12"/>
     </row>
     <row r="16" spans="1:9" ht="12.75">
@@ -1244,7 +1274,7 @@
         <v>31</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C17" s="15" t="str">
         <f>TPE!C7</f>
@@ -1255,11 +1285,13 @@
         <v>SM, SE, Engineer, PC, PPC, Rigging Eng</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F17" s="15"/>
       <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
+      <c r="H17" s="16" t="s">
+        <v>187</v>
+      </c>
       <c r="I17" s="12"/>
     </row>
     <row r="18" spans="1:9" ht="12.75">
@@ -1286,7 +1318,7 @@
         <v>52</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C19" s="15" t="str">
         <f>TPE!C9</f>
@@ -1297,13 +1329,17 @@
         <v>semua HSE (koordinator dan tiap lokasi). HSE Manager hanya bila tertulis "HSE Manager"</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F19" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15"/>
+      <c r="G19" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="H19" s="16" t="s">
+        <v>188</v>
+      </c>
       <c r="I19" s="12"/>
     </row>
     <row r="20" spans="1:9" ht="12.75">
@@ -1330,7 +1366,7 @@
         <v>41</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C21" s="15" t="str">
         <f>TPE!C11</f>
@@ -1344,10 +1380,12 @@
         <v>41</v>
       </c>
       <c r="F21" s="16" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G21" s="15"/>
-      <c r="H21" s="15"/>
+      <c r="H21" s="16" t="s">
+        <v>189</v>
+      </c>
       <c r="I21" s="12"/>
     </row>
     <row r="22" spans="1:9" ht="12.75">
@@ -1371,7 +1409,7 @@
     </row>
     <row r="23" spans="1:9" ht="12.75">
       <c r="A23" s="13" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B23" s="14"/>
       <c r="C23" s="15" t="str">
@@ -1390,10 +1428,10 @@
     </row>
     <row r="24" spans="1:9" ht="25.5">
       <c r="A24" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C24" s="15" t="str">
         <f>TPE!C14</f>
@@ -1407,15 +1445,19 @@
         <v>36</v>
       </c>
       <c r="F24" s="16" t="s">
-        <v>184</v>
-      </c>
-      <c r="G24" s="15"/>
-      <c r="H24" s="15"/>
+        <v>182</v>
+      </c>
+      <c r="G24" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="H24" s="16" t="s">
+        <v>190</v>
+      </c>
       <c r="I24" s="12"/>
     </row>
     <row r="25" spans="1:9" ht="12.75">
       <c r="A25" s="13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B25" s="14"/>
       <c r="C25" s="15"/>
@@ -1434,7 +1476,7 @@
         <v>43</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C26" s="15" t="str">
         <f>TPE!C18</f>
@@ -1445,10 +1487,10 @@
         <v>semua SPV</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F26" s="16" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G26" s="15"/>
       <c r="H26" s="15"/>
@@ -1461,7 +1503,7 @@
         <v>47</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C27" s="15" t="str">
         <f>TPE!C19</f>
@@ -1474,12 +1516,14 @@
       <c r="E27" s="15"/>
       <c r="F27" s="15"/>
       <c r="G27" s="15"/>
-      <c r="H27" s="15"/>
+      <c r="H27" s="16" t="s">
+        <v>47</v>
+      </c>
       <c r="I27" s="12"/>
     </row>
-    <row r="28" spans="1:9" ht="25.5">
+    <row r="28" spans="1:9" ht="12.75">
       <c r="A28" s="13" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B28" s="14"/>
       <c r="C28" s="15" t="str">
@@ -1496,9 +1540,9 @@
       <c r="H28" s="15"/>
       <c r="I28" s="12"/>
     </row>
-    <row r="29" spans="1:9" ht="25.5">
+    <row r="29" spans="1:9" ht="12.75">
       <c r="A29" s="13" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B29" s="14"/>
       <c r="C29" s="15" t="str">
@@ -1515,9 +1559,9 @@
       <c r="H29" s="15"/>
       <c r="I29" s="12"/>
     </row>
-    <row r="30" spans="1:9" ht="25.5">
+    <row r="30" spans="1:9" ht="12.75">
       <c r="A30" s="13" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B30" s="14"/>
       <c r="C30" s="15" t="str">
@@ -1550,21 +1594,23 @@
         <v>Inspector Scaffolding, Scaffolder, anggota Team Scaffolder tanpa role</v>
       </c>
       <c r="E31" s="16" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F31" s="16" t="s">
         <v>50</v>
       </c>
       <c r="G31" s="15"/>
-      <c r="H31" s="15"/>
+      <c r="H31" s="16" t="s">
+        <v>191</v>
+      </c>
       <c r="I31" s="12"/>
     </row>
     <row r="32" spans="1:9" ht="38.25">
       <c r="A32" s="13" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C32" s="15" t="str">
         <f>TPE!C24</f>
@@ -1575,21 +1621,23 @@
         <v>Teknisi, Rigger, Welder, Skill, Helper, Fitter</v>
       </c>
       <c r="E32" s="16" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F32" s="16" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G32" s="15"/>
-      <c r="H32" s="15"/>
+      <c r="H32" s="16" t="s">
+        <v>192</v>
+      </c>
       <c r="I32" s="12"/>
     </row>
     <row r="33" spans="1:9" ht="51">
       <c r="A33" s="13" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C33" s="15" t="str">
         <f>TPE!C25</f>
@@ -1600,18 +1648,20 @@
         <v>Helper/anggota lokasi Warehouse</v>
       </c>
       <c r="E33" s="16" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F33" s="16" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G33" s="15"/>
-      <c r="H33" s="15"/>
+      <c r="H33" s="16" t="s">
+        <v>113</v>
+      </c>
       <c r="I33" s="12"/>
     </row>
-    <row r="34" spans="1:9" ht="25.5">
+    <row r="34" spans="1:9" ht="12.75">
       <c r="A34" s="13" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B34" s="14"/>
       <c r="C34" s="15" t="str">
@@ -1633,7 +1683,7 @@
         <v>59</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C35" s="15" t="str">
         <f>TPE!C27</f>
@@ -1644,18 +1694,22 @@
         <v>Admin, DOCON, Matecon / Matkon (material control)</v>
       </c>
       <c r="E35" s="16" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F35" s="16" t="s">
-        <v>185</v>
-      </c>
-      <c r="G35" s="15"/>
-      <c r="H35" s="15"/>
+        <v>183</v>
+      </c>
+      <c r="G35" s="16" t="s">
+        <v>195</v>
+      </c>
+      <c r="H35" s="16" t="s">
+        <v>193</v>
+      </c>
       <c r="I35" s="12"/>
     </row>
     <row r="36" spans="1:9" ht="25.5">
       <c r="A36" s="13" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B36" s="14" t="s">
         <v>63</v>
@@ -1671,10 +1725,12 @@
       <c r="E36" s="15"/>
       <c r="F36" s="15"/>
       <c r="G36" s="15"/>
-      <c r="H36" s="15"/>
+      <c r="H36" s="16" t="s">
+        <v>63</v>
+      </c>
       <c r="I36" s="12"/>
     </row>
-    <row r="37" spans="1:9" ht="25.5">
+    <row r="37" spans="1:9" ht="38.25">
       <c r="A37" s="13" t="s">
         <v>73</v>
       </c>
@@ -1685,13 +1741,13 @@
       <c r="F37" s="12"/>
       <c r="G37" s="12"/>
       <c r="H37" s="12"/>
-      <c r="I37" s="15" t="s">
-        <v>74</v>
+      <c r="I37" s="16" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="15.75" customHeight="1">
       <c r="A38" s="13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B38" s="17"/>
       <c r="C38" s="12"/>
@@ -1700,107 +1756,107 @@
       <c r="F38" s="12"/>
       <c r="G38" s="12"/>
       <c r="H38" s="12"/>
-      <c r="I38" s="15" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9">
+      <c r="I38" s="16" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="12.75">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
     </row>
-    <row r="40" spans="1:9">
+    <row r="40" spans="1:9" ht="12.75">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
     </row>
-    <row r="41" spans="1:9">
+    <row r="41" spans="1:9" ht="12.75">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
     </row>
-    <row r="42" spans="1:9">
+    <row r="42" spans="1:9" ht="12.75">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
     </row>
-    <row r="43" spans="1:9">
+    <row r="43" spans="1:9" ht="12.75">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
     </row>
-    <row r="44" spans="1:9">
+    <row r="44" spans="1:9" ht="12.75">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
     </row>
-    <row r="45" spans="1:9">
+    <row r="45" spans="1:9" ht="12.75">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
     </row>
-    <row r="46" spans="1:9">
+    <row r="46" spans="1:9" ht="12.75">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
     </row>
-    <row r="47" spans="1:9">
+    <row r="47" spans="1:9" ht="12.75">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
     </row>
-    <row r="48" spans="1:9">
+    <row r="48" spans="1:9" ht="12.75">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
     </row>
-    <row r="49" spans="1:2">
+    <row r="49" spans="1:2" ht="12.75">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
     </row>
-    <row r="50" spans="1:2">
+    <row r="50" spans="1:2" ht="12.75">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
     </row>
-    <row r="51" spans="1:2">
+    <row r="51" spans="1:2" ht="12.75">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
     </row>
-    <row r="52" spans="1:2">
+    <row r="52" spans="1:2" ht="12.75">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
     </row>
-    <row r="53" spans="1:2">
+    <row r="53" spans="1:2" ht="12.75">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
     </row>
-    <row r="54" spans="1:2">
+    <row r="54" spans="1:2" ht="12.75">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
     </row>
-    <row r="55" spans="1:2">
+    <row r="55" spans="1:2" ht="12.75">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
     </row>
-    <row r="56" spans="1:2">
+    <row r="56" spans="1:2" ht="12.75">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
     </row>
-    <row r="57" spans="1:2">
+    <row r="57" spans="1:2" ht="12.75">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
     </row>
-    <row r="58" spans="1:2">
+    <row r="58" spans="1:2" ht="12.75">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
     </row>
-    <row r="59" spans="1:2">
+    <row r="59" spans="1:2" ht="12.75">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
     </row>
-    <row r="63" spans="1:2">
+    <row r="63" spans="1:2" ht="12.75">
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
     </row>
-    <row r="64" spans="1:2">
+    <row r="64" spans="1:2" ht="12.75">
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
     </row>
-    <row r="65" spans="1:2">
+    <row r="65" spans="1:2" ht="12.75">
       <c r="A65" s="1"/>
       <c r="B65" s="1"/>
     </row>
-    <row r="66" spans="1:2">
+    <row r="66" spans="1:2" ht="12.75">
       <c r="A66" s="1"/>
       <c r="B66" s="1"/>
     </row>
@@ -1996,15 +2052,15 @@
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>38</v>
@@ -2019,40 +2075,40 @@
         <v>2</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B15" s="1"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
       <c r="K15" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B16" s="1"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
       <c r="K16" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B17" s="1"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
       <c r="K17" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -2087,38 +2143,38 @@
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="K20" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
       <c r="K21" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
       <c r="K22" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -2158,7 +2214,7 @@
         <v>11</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -2178,18 +2234,18 @@
         <v>5</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="26" spans="1:11">
       <c r="A26" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B26" s="1"/>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
       <c r="K26" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -2207,7 +2263,7 @@
     </row>
     <row r="28" spans="1:11">
       <c r="A28" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>64</v>
@@ -2215,12 +2271,12 @@
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
       <c r="K28" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C30" s="1">
         <f>SUM(C3:C28)</f>
@@ -2251,7 +2307,7 @@
     <col min="1" max="1" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" ht="12.75">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -2272,12 +2328,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" ht="12.75">
       <c r="A2" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" ht="12.75">
       <c r="A3" s="1" t="s">
         <v>17</v>
       </c>
@@ -2291,13 +2347,13 @@
         <v>sm</v>
       </c>
       <c r="H3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="12.75">
       <c r="A4" s="1" t="s">
         <v>21</v>
       </c>
@@ -2310,18 +2366,18 @@
         <v>se</v>
       </c>
       <c r="H4" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" ht="12.75">
       <c r="A5" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C5" t="str" cm="1">
         <f t="array" ref="C5">IFERROR(_xlfn.TEXTJOIN(", ", TRUE, _xlfn._xlws.FILTER($H$3:$H$33, $I$3:$I$33 = B5)),"")</f>
@@ -2337,7 +2393,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" ht="12.75">
       <c r="A6" s="1" t="s">
         <v>37</v>
       </c>
@@ -2356,7 +2412,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" ht="12.75">
       <c r="A7" s="1" t="s">
         <v>31</v>
       </c>
@@ -2374,13 +2430,13 @@
         <v>hse</v>
       </c>
       <c r="H7" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="I7" s="4" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" ht="12.75">
       <c r="A8" s="1" t="s">
         <v>48</v>
       </c>
@@ -2393,13 +2449,13 @@
         <v>staff</v>
       </c>
       <c r="H8" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" ht="12.75">
       <c r="A9" s="1" t="s">
         <v>52</v>
       </c>
@@ -2417,13 +2473,13 @@
         <v>skilled</v>
       </c>
       <c r="H9" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="I9" s="4" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" ht="12.75">
       <c r="A10" s="1" t="s">
         <v>65</v>
       </c>
@@ -2436,13 +2492,13 @@
         <v>scf</v>
       </c>
       <c r="H10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="I10" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" ht="12.75">
       <c r="A11" s="1" t="s">
         <v>41</v>
       </c>
@@ -2466,7 +2522,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" ht="12.75">
       <c r="A12" s="1" t="s">
         <v>69</v>
       </c>
@@ -2478,15 +2534,15 @@
         <v>fore</v>
       </c>
       <c r="H12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="12.75">
       <c r="A13" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C13" t="str" cm="1">
         <f t="array" ref="C13">IFERROR(_xlfn.TEXTJOIN(", ", TRUE, _xlfn._xlws.FILTER($H$3:$H$33, $I$3:$I$33 = B13)),"")</f>
@@ -2496,15 +2552,15 @@
         <v>labor</v>
       </c>
       <c r="H13" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="12.75">
       <c r="A14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>57</v>
@@ -2520,15 +2576,15 @@
         <v>operator</v>
       </c>
       <c r="H14" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="12.75">
       <c r="A15" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" t="str" cm="1">
@@ -2536,15 +2592,15 @@
         <v/>
       </c>
       <c r="H15" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="12.75">
       <c r="A16" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B16" s="1"/>
       <c r="C16" t="str" cm="1">
@@ -2552,15 +2608,15 @@
         <v/>
       </c>
       <c r="H16" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="12.75">
       <c r="A17" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" t="str" cm="1">
@@ -2568,13 +2624,13 @@
         <v/>
       </c>
       <c r="H17" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="12.75">
       <c r="A18" s="1" t="s">
         <v>43</v>
       </c>
@@ -2589,33 +2645,33 @@
         <v>2</v>
       </c>
       <c r="H18" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="12.75">
       <c r="A19" s="1" t="s">
         <v>47</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C19" t="str" cm="1">
         <f t="array" ref="C19">IFERROR(_xlfn.TEXTJOIN(", ", TRUE, _xlfn._xlws.FILTER($H$3:$H$33, $I$3:$I$33 = B19)),"")</f>
         <v>FM ELEC, FM FT, FM MW</v>
       </c>
       <c r="H19" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="12.75">
       <c r="A20" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" t="str" cm="1">
@@ -2623,15 +2679,15 @@
         <v/>
       </c>
       <c r="H20" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="12.75">
       <c r="A21" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" t="str" cm="1">
@@ -2639,15 +2695,15 @@
         <v/>
       </c>
       <c r="H21" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="12.75">
       <c r="A22" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B22" s="1"/>
       <c r="C22" t="str" cm="1">
@@ -2655,18 +2711,18 @@
         <v/>
       </c>
       <c r="H22" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="I22" s="4" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" ht="12.75">
       <c r="A23" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C23" t="str" cm="1">
         <f t="array" ref="C23">IFERROR(_xlfn.TEXTJOIN(", ", TRUE, _xlfn._xlws.FILTER($H$3:$H$33, $I$3:$I$33 = B23)),"")</f>
@@ -2676,18 +2732,18 @@
         <v>11</v>
       </c>
       <c r="H23" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="12.75">
       <c r="A24" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C24" t="str" cm="1">
         <f t="array" ref="C24">IFERROR(_xlfn.TEXTJOIN(", ", TRUE, _xlfn._xlws.FILTER($H$3:$H$33, $I$3:$I$33 = B24)),"")</f>
@@ -2697,18 +2753,18 @@
         <v>36</v>
       </c>
       <c r="H24" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="12.75">
       <c r="A25" s="1" t="s">
         <v>55</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C25" t="str" cm="1">
         <f t="array" ref="C25">IFERROR(_xlfn.TEXTJOIN(", ", TRUE, _xlfn._xlws.FILTER($H$3:$H$33, $I$3:$I$33 = B25)),"")</f>
@@ -2718,15 +2774,15 @@
         <v>1</v>
       </c>
       <c r="H25" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="12.75">
       <c r="A26" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" t="str" cm="1">
@@ -2734,18 +2790,18 @@
         <v/>
       </c>
       <c r="H26" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="12.75">
       <c r="A27" s="1" t="s">
         <v>59</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C27" t="str" cm="1">
         <f t="array" ref="C27">IFERROR(_xlfn.TEXTJOIN(", ", TRUE, _xlfn._xlws.FILTER($H$3:$H$33, $I$3:$I$33 = B27)),"")</f>
@@ -2755,33 +2811,33 @@
         <v>3</v>
       </c>
       <c r="H27" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="12.75">
       <c r="A28" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C28" t="str" cm="1">
         <f t="array" ref="C28">IFERROR(_xlfn.TEXTJOIN(", ", TRUE, _xlfn._xlws.FILTER($H$3:$H$33, $I$3:$I$33 = B28)),"")</f>
         <v>OPR CRANE, OPR TMC</v>
       </c>
       <c r="H28" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="12.75">
       <c r="A29" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C29" s="1"/>
       <c r="E29" s="1">
@@ -2789,42 +2845,42 @@
         <v>64</v>
       </c>
       <c r="H29" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="15.75" customHeight="1">
       <c r="H30" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="15.75" customHeight="1">
       <c r="H31" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="15.75" customHeight="1">
       <c r="H32" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="33" spans="8:9" ht="15.75" customHeight="1">
       <c r="H33" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -2847,11 +2903,11 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="8" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
@@ -2875,7 +2931,7 @@
         <v>18</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="10" t="s">
@@ -2893,7 +2949,7 @@
         <v>23</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D4" s="7"/>
       <c r="E4" s="10" t="s">
@@ -2929,7 +2985,7 @@
         <v>39</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D6" s="7"/>
       <c r="E6" s="10" t="s">
@@ -2947,7 +3003,7 @@
         <v>30</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D7" s="7"/>
       <c r="E7" s="10" t="s">
@@ -2965,7 +3021,7 @@
         <v>49</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D8" s="7"/>
       <c r="E8" s="10" t="s">
@@ -2983,7 +3039,7 @@
         <v>46</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D9" s="7"/>
       <c r="E9" s="10" t="s">
@@ -3001,7 +3057,7 @@
         <v>60</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D10" s="7"/>
       <c r="E10" s="10" t="s">
@@ -3019,7 +3075,7 @@
         <v>66</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D11" s="7"/>
       <c r="E11" s="10" t="s">
@@ -3037,7 +3093,7 @@
         <v>71</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D12" s="7"/>
       <c r="E12" s="10" t="s">
@@ -3049,17 +3105,17 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D13" s="7"/>
       <c r="E13" s="10" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F13" s="10" t="s">
         <v>68</v>
@@ -3067,17 +3123,17 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>57</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D14" s="7"/>
       <c r="E14" s="10" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F14" s="10" t="s">
         <v>68</v>
@@ -3085,47 +3141,47 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="10" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D15" s="7"/>
       <c r="E15" s="10" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="10" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B16" s="7"/>
       <c r="C16" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D16" s="7"/>
       <c r="E16" s="10" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="10" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D17" s="7"/>
       <c r="E17" s="10" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F17" s="10" t="s">
         <v>68</v>
@@ -3139,11 +3195,11 @@
         <v>68</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D18" s="7"/>
       <c r="E18" s="10" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F18" s="10" t="s">
         <v>68</v>
@@ -3154,67 +3210,67 @@
         <v>47</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D19" s="7"/>
       <c r="E19" s="10" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="10" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D20" s="7"/>
       <c r="E20" s="10" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="10" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D21" s="7"/>
       <c r="E21" s="10" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="10" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D22" s="7"/>
       <c r="E22" s="10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -3222,69 +3278,69 @@
         <v>50</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C23" s="7" t="s">
         <v>50</v>
       </c>
       <c r="D23" s="7"/>
       <c r="E23" s="10" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="10" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D24" s="7"/>
       <c r="E24" s="10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="10" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D25" s="7"/>
       <c r="E25" s="10" t="s">
         <v>50</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="10" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D26" s="7"/>
       <c r="E26" s="10" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -3292,35 +3348,35 @@
         <v>59</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D27" s="7"/>
       <c r="E27" s="10" t="s">
         <v>63</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="10" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C28" s="7" t="s">
         <v>63</v>
       </c>
       <c r="D28" s="7"/>
       <c r="E28" s="10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -3329,7 +3385,7 @@
       <c r="C29" s="7"/>
       <c r="D29" s="7"/>
       <c r="E29" s="10" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F29" s="10" t="s">
         <v>66</v>
@@ -3341,10 +3397,10 @@
       <c r="C30" s="7"/>
       <c r="D30" s="7"/>
       <c r="E30" s="10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -3353,10 +3409,10 @@
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
       <c r="E31" s="10" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F31" s="10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -3365,10 +3421,10 @@
       <c r="C32" s="7"/>
       <c r="D32" s="7"/>
       <c r="E32" s="10" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F32" s="10" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="33" spans="3:5">
@@ -3532,7 +3588,7 @@
     <col min="1" max="1" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" ht="12.75">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -3555,12 +3611,12 @@
         <v>46287</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" ht="12.75">
       <c r="A2" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" ht="12.75">
       <c r="A3" s="1" t="s">
         <v>17</v>
       </c>
@@ -3572,7 +3628,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" ht="12.75">
       <c r="A4" s="1" t="s">
         <v>21</v>
       </c>
@@ -3586,7 +3642,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" ht="12.75">
       <c r="A5" s="1" t="s">
         <v>26</v>
       </c>
@@ -3597,10 +3653,10 @@
         <v>1</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="12.75">
       <c r="A6" s="1" t="s">
         <v>37</v>
       </c>
@@ -3611,7 +3667,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" ht="12.75">
       <c r="A7" s="1" t="s">
         <v>31</v>
       </c>
@@ -3622,10 +3678,10 @@
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="12.75">
       <c r="A8" s="1" t="s">
         <v>52</v>
       </c>
@@ -3636,12 +3692,12 @@
         <v>6</v>
       </c>
       <c r="H8" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="12.75">
       <c r="A9" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>38</v>
@@ -3650,10 +3706,10 @@
         <v>9</v>
       </c>
       <c r="H9" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="12.75">
       <c r="A10" s="1" t="s">
         <v>41</v>
       </c>
@@ -3661,10 +3717,10 @@
         <v>42</v>
       </c>
       <c r="H10" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="12.75">
       <c r="A11" s="1" t="s">
         <v>43</v>
       </c>
@@ -3675,10 +3731,10 @@
         <v>5</v>
       </c>
       <c r="H11" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="12.75">
       <c r="A12" s="1" t="s">
         <v>47</v>
       </c>
@@ -3689,10 +3745,10 @@
         <v>2</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="12.75">
       <c r="A13" s="1" t="s">
         <v>50</v>
       </c>
@@ -3703,12 +3759,12 @@
         <v>2</v>
       </c>
       <c r="H13" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="12.75">
       <c r="A14" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>54</v>
@@ -3717,12 +3773,12 @@
         <v>3</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="12.75">
       <c r="A15" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>56</v>
@@ -3731,10 +3787,10 @@
         <v>2</v>
       </c>
       <c r="H15" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="12.75">
       <c r="A16" s="1" t="s">
         <v>59</v>
       </c>
@@ -3745,12 +3801,12 @@
         <v>6</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="12.75">
       <c r="A17" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>64</v>
@@ -3759,12 +3815,12 @@
         <v>1</v>
       </c>
       <c r="H17" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="12.75">
       <c r="A19" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F19" s="1">
         <v>108</v>
@@ -3772,10 +3828,10 @@
     </row>
     <row r="26" spans="1:8" ht="15.75" customHeight="1">
       <c r="B26" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C26" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="15.75" customHeight="1">
@@ -3783,7 +3839,7 @@
         <v>31</v>
       </c>
       <c r="C27" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="15.75" customHeight="1">
@@ -3791,7 +3847,7 @@
         <v>52</v>
       </c>
       <c r="C28" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="15.75" customHeight="1">
@@ -3799,23 +3855,23 @@
         <v>41</v>
       </c>
       <c r="C29" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="15.75" customHeight="1">
       <c r="B30" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C30" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="15.75" customHeight="1">
       <c r="B31" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C31" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="15.75" customHeight="1">
@@ -3823,7 +3879,7 @@
         <v>59</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="33" spans="2:3" ht="15.75" customHeight="1">
@@ -3831,7 +3887,7 @@
         <v>43</v>
       </c>
       <c r="C33" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="34" spans="2:3" ht="15.75" customHeight="1">
@@ -3839,7 +3895,7 @@
         <v>47</v>
       </c>
       <c r="C34" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="35" spans="2:3" ht="15.75" customHeight="1">
@@ -3847,15 +3903,15 @@
         <v>50</v>
       </c>
       <c r="C35" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="36" spans="2:3" ht="15.75" customHeight="1">
       <c r="B36" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C36" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="37" spans="2:3" ht="15.75" customHeight="1">
@@ -3863,15 +3919,15 @@
         <v>55</v>
       </c>
       <c r="C37" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="38" spans="2:3" ht="15.75" customHeight="1">
       <c r="B38" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C38" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -3889,7 +3945,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>3</v>
@@ -4043,7 +4099,7 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F19" s="1">
         <v>34</v>

</xml_diff>